<commit_message>
Final tests, some source code changes
</commit_message>
<xml_diff>
--- a/docs/סיכום_טסטים.xlsx
+++ b/docs/סיכום_טסטים.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hwath\Codes\VisualStudio\IronGate\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2483C94-E032-4228-BA6D-C8ED93178D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFCCE267-B26A-487B-A408-A571D2FF2415}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{8B486C0D-BB0B-425A-AA9A-D44437056338}"/>
   </bookViews>
@@ -337,7 +337,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1202,34 +1202,34 @@
       <c r="AH10" s="7"/>
     </row>
     <row r="11" spans="1:34" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G11" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="H11" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="I11" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="J11" s="8" t="s">
+      <c r="E11" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="J11" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1266,34 +1266,34 @@
       </c>
     </row>
     <row r="13" spans="1:34" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E13" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G13" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="I13" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="J13" s="8" t="s">
+      <c r="E13" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="J13" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1362,98 +1362,98 @@
       </c>
     </row>
     <row r="16" spans="1:34" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G16" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="H16" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="I16" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="J16" s="8" t="s">
+      <c r="E16" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="J16" s="5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E17" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G17" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="I17" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="J17" s="8" t="s">
+      <c r="E17" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="J17" s="5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E18" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G18" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="H18" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="I18" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="J18" s="8" t="s">
+      <c r="E18" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G18" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="J18" s="5" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1586,66 +1586,66 @@
       </c>
     </row>
     <row r="23" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="8" t="s">
+      <c r="A23" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D23" s="8" t="s">
+      <c r="D23" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E23" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F23" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G23" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="H23" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="I23" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="J23" s="8" t="s">
+      <c r="E23" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="J23" s="5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="8" t="s">
+      <c r="A24" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E24" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F24" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G24" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="H24" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="I24" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="J24" s="8" t="s">
+      <c r="E24" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="J24" s="5" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added powerpoint presentation and a few bug fixes
</commit_message>
<xml_diff>
--- a/docs/סיכום_טסטים.xlsx
+++ b/docs/סיכום_טסטים.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hwath\Codes\VisualStudio\IronGate\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFCCE267-B26A-487B-A408-A571D2FF2415}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75AF68A3-C489-4C35-BB65-A68E89A9AE69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{8B486C0D-BB0B-425A-AA9A-D44437056338}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="טבלת סיכום תוצאות" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tests!$B$1:$J$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tests!$B$1:$J$21</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="64">
   <si>
     <t>ID</t>
   </si>
@@ -113,9 +113,6 @@
   </si>
   <si>
     <t>on</t>
-  </si>
-  <si>
-    <t>Rate limit vs password strength</t>
   </si>
   <si>
     <t>Spray under rate limit</t>
@@ -200,15 +197,9 @@
     <t>test08</t>
   </si>
   <si>
-    <t>test09</t>
-  </si>
-  <si>
     <t>test10</t>
   </si>
   <si>
-    <t>test11</t>
-  </si>
-  <si>
     <t>test12</t>
   </si>
   <si>
@@ -239,48 +230,10 @@
     <t>test20</t>
   </si>
   <si>
-    <t>Medium + brute force: sha256 vs bcrypt vs argon2id
-Run: test07 vs test08 vs test09
-Look for: TTFC, compromises %, attempts/sec, server latency/CPU. This is your cleanest “hash choice matters online” story.
-Easy + brute force: sha256 vs bcrypt vs argon2id
-Run: test01 vs test03 vs test05
-Look for: how quickly each falls when there are no defenses, and how much compute cost alone slows the attacker.
-Pepper effect on online attacks (sanity check)
-Run: test01 vs test02, test03 vs test04, test05 vs test06
-Look for: verify cost should be near-identical; success rates should match. If they don’t, pepper is being applied inconsistently.
-Brute force vs password spraying under rate limit
-Run: test10 vs test12 (same hash, same RL)
-Look for: spray often avoids per-user RL bottlenecks better; compare compromises-per-minute and 429 rates.
-Brute force vs password spraying under full stack defenses
-Run: test18 vs test20
-Look for: whether captcha/lockout triggers earlier for one attack style; which yields higher compromises before “attack stops”.
-Captcha-only: brute force vs spray
-Run: test15 vs test16
-Look for: consecutive-failure captcha can be “reset” by spraying patterns; measure captcha prompts per successful login.
-Rate limit only vs lockout only (same hash/inputs)
-Run: test10 vs test13
-Look for: RL throttles but keeps accounts available; lockout can terminate quickly but may create a DoS vector (lots of lockouts).
-Medium users: no defenses vs rate limit vs lockout vs captcha
-Run: test07 vs test11 vs test14 vs test17
-Look for: which control actually changes compromise probability vs just slowing the attacker.
-Full stack: argon2id+pepper vs sha256+pepper (defenses held constant)
-Run: test18 vs test19
-Look for: whether heavy hashing meaningfully improves outcome once RL/lockout/captcha already dominate.
-Server-stability comparison: argon2id vs bcrypt under sustained attack
-Run: test05 vs test03 
-Look for: response time spikes, error rates, and whether the “stronger” hash causes availability issues under load.</t>
-  </si>
-  <si>
-    <t>test21</t>
-  </si>
-  <si>
     <t>test22</t>
   </si>
   <si>
     <t>test23</t>
-  </si>
-  <si>
-    <t>HARD_ONLY</t>
   </si>
 </sst>
 </file>
@@ -316,7 +269,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -332,12 +285,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -369,7 +316,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -391,9 +338,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -709,7 +653,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82F8A593-C5C9-4B44-AE84-7E1661D577D0}">
-  <dimension ref="A1:AH24"/>
+  <dimension ref="A1:AH21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -742,18 +686,18 @@
         <v>5</v>
       </c>
       <c r="H1" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J1" s="4" t="s">
         <v>41</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:34" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>9</v>
@@ -785,7 +729,7 @@
     </row>
     <row r="3" spans="1:34" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>14</v>
@@ -814,9 +758,7 @@
       <c r="J3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="O3" s="7" t="s">
-        <v>65</v>
-      </c>
+      <c r="O3" s="7"/>
       <c r="P3" s="7"/>
       <c r="Q3" s="7"/>
       <c r="R3" s="7"/>
@@ -839,7 +781,7 @@
     </row>
     <row r="4" spans="1:34" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>9</v>
@@ -891,7 +833,7 @@
     </row>
     <row r="5" spans="1:34" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>16</v>
@@ -943,7 +885,7 @@
     </row>
     <row r="6" spans="1:34" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>9</v>
@@ -995,7 +937,7 @@
     </row>
     <row r="7" spans="1:34" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>18</v>
@@ -1047,7 +989,7 @@
     </row>
     <row r="8" spans="1:34" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>19</v>
@@ -1099,7 +1041,7 @@
     </row>
     <row r="9" spans="1:34" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>19</v>
@@ -1150,133 +1092,113 @@
       <c r="AH9" s="7"/>
     </row>
     <row r="10" spans="1:34" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="8" t="s">
+      <c r="A10" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="G10" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="I10" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="O10" s="7"/>
-      <c r="P10" s="7"/>
-      <c r="Q10" s="7"/>
-      <c r="R10" s="7"/>
-      <c r="S10" s="7"/>
-      <c r="T10" s="7"/>
-      <c r="U10" s="7"/>
-      <c r="V10" s="7"/>
-      <c r="W10" s="7"/>
-      <c r="X10" s="7"/>
-      <c r="Y10" s="7"/>
-      <c r="Z10" s="7"/>
-      <c r="AA10" s="7"/>
-      <c r="AB10" s="7"/>
-      <c r="AC10" s="7"/>
-      <c r="AD10" s="7"/>
-      <c r="AE10" s="7"/>
-      <c r="AF10" s="7"/>
-      <c r="AG10" s="7"/>
-      <c r="AH10" s="7"/>
+      <c r="D10" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="11" spans="1:34" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:34" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="5" t="s">
+      <c r="B12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D12" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G11" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="J11" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:34" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G12" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="H12" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="I12" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="J12" s="8" t="s">
+      <c r="E12" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="J12" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>21</v>
@@ -1288,10 +1210,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="J13" s="5" t="s">
         <v>13</v>
@@ -1299,10 +1221,10 @@
     </row>
     <row r="14" spans="1:34" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>10</v>
@@ -1323,24 +1245,24 @@
         <v>13</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:34" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>21</v>
@@ -1355,24 +1277,24 @@
         <v>13</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:34" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>10</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>21</v>
@@ -1395,48 +1317,48 @@
     </row>
     <row r="17" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G17" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="J17" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>60</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>10</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>21</v>
@@ -1445,13 +1367,13 @@
         <v>12</v>
       </c>
       <c r="G18" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="J18" s="5" t="s">
         <v>24</v>
@@ -1465,10 +1387,10 @@
         <v>34</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>21</v>
@@ -1489,18 +1411,18 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>21</v>
@@ -1508,14 +1430,14 @@
       <c r="F20" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="G20" s="5" t="b">
-        <v>1</v>
+      <c r="G20" s="5" t="s">
+        <v>24</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="J20" s="5" t="s">
         <v>24</v>
@@ -1523,140 +1445,44 @@
     </row>
     <row r="21" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C21" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>28</v>
-      </c>
       <c r="E21" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G21" s="5" t="b">
-        <v>1</v>
+        <v>12</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>24</v>
       </c>
       <c r="H21" s="5" t="s">
         <v>24</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="J21" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D22" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F22" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G22" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="H22" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="I22" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="J22" s="8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F23" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H23" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="I23" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="J23" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G24" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H24" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="I24" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="J24" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="B1:J24" xr:uid="{82F8A593-C5C9-4B44-AE84-7E1661D577D0}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:J10">
+  <autoFilter ref="B1:J21" xr:uid="{82F8A593-C5C9-4B44-AE84-7E1661D577D0}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:J9">
       <sortCondition descending="1" ref="H1"/>
     </sortState>
   </autoFilter>
   <mergeCells count="1">
-    <mergeCell ref="O3:AH10"/>
+    <mergeCell ref="O3:AH9"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1677,19 +1503,19 @@
   <sheetData>
     <row r="1" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">

</xml_diff>